<commit_message>
analysis: Step 2 human benchmark v2 — Fawkner Visium, Fawkner+Burclaff, Gao+Wang
Three new human fetal-vs-adult contrasts benchmarked on the 31 Step 1 markers
under the frozen qualification rule (5c3bcef). H-new2 is the only qualifying
human contrast; no signature is built. Dataset registry and 31-marker summary
updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not used or deferred'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -106,10 +106,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Invalidated with Step 2</t>
+          <t>Invalidated with Step 2; fetal arm reused in benchmark v2 (H-new3, Gao-original recomputed)</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Replacement candidate, human</t>
+          <t>Replacement candidate, human; fetal arm of H-new2 (v2)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -938,22 +938,22 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>10x scRNA-seq, raw UMI (GPL15520/GPL18573/GPL24676)</t>
+          <t>10x scRNA-seq, raw UMI, hashtag-multiplexed pools (GPL15520/GPL18573/GPL24676)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Fetal EpCAM+ epithelium only; no adult arm</t>
+          <t>v1: fetal EpCAM+ detection only; v2: hashtag-demultiplexed fetal samples vs Burclaff adult (H-new2)</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>4 fetal pools</t>
+          <t>v1: 4 pools; v2: 22 fetal hashtag samples</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Fetal-expression annotation only; no fetal/adult FC possible</t>
+          <t>GEO GEX/HTO pairing corrected by barcode overlap; hashtag samples can share a fetus</t>
         </is>
       </c>
     </row>
@@ -1094,37 +1094,37 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2 (benchmark v2)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>T1 bulk tumour support</t>
+          <t>H-new1 human fetal + adult, same study</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>TCGA COAD + READ</t>
+          <t>Fawkner-Corbett Visium</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Cancer Genome Atlas Network</t>
+          <t>Fawkner-Corbett D et al.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Nature, 2012</t>
+          <t>Cell, 2021</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>22810696</t>
+          <t>33406409</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>10.1038/nature11252</t>
+          <t>10.1016/j.cell.2020.12.016</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1134,64 +1134,64 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>TCGA-COAD, TCGA-READ (GDC) via recount3</t>
+          <t>GSE158328</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Bulk RNA-seq, recount3 Monorail, GENCODE v26 read counts</t>
+          <t>10x Visium spatial, raw counts (GPL18573)</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Primary tumour vs solid-tissue normal, ~ tissue + project</t>
+          <t>Epithelial-rich spots (top quartile epithelial score, EPCAM+) pseudobulked per section; fetal vs adult, ~ stage</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>624 tumours (458 COAD, 166 READ) / 51 normals</t>
+          <t>6 fetal sections (2 colon, 4 SI) / 2 adult colon sections</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>bulk_support annotation (no veto, plan v2)</t>
+          <t>Adult n = 2 sections; fetal spots markedly less epithelial (composition confound)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2 (benchmark v2)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>T1 sensitivity</t>
+          <t>H-new2 adult reference</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>GTEx v8 colon</t>
+          <t>Burclaff adult epithelium</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>GTEx Consortium</t>
+          <t>Burclaff J et al.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Science, 2020</t>
+          <t>Cell Mol Gastroenterol Hepatol, 2022</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>32913098</t>
+          <t>35176508</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>10.1126/science.aaz1776</t>
+          <t>10.1016/j.jcmgh.2022.02.007</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1201,233 +1201,434 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>GTEx v8 (dbGaP phs000424) via recount3</t>
+          <t>GSE185224</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Bulk RNA-seq, same recount3 pipeline</t>
+          <t>10x scRNA-seq, raw counts (annotated h5ad, GPL18573)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>TCGA tumour vs GTEx Colon – Transverse; direction only (source confounded)</t>
+          <t>Healthy adult epithelium, 6 regions, pseudobulk per donor; vs Fawkner fetal scRNA (study confounded with stage)</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>433 GTEx / 624 tumours</t>
+          <t>3 adult donors</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>Descriptive only</t>
+          <t>12,590 epithelial cells</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>2 (benchmark v2)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>H-new3 adult reference</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Wang adult ileum/colon/rectum</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Wang Y et al.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>J Exp Med, 2020</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>31753849</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>10.1084/jem.20191130</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>GSE125970</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>10x scRNA-seq, raw UMI (GPL20795)</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Adult epithelium per sample; vs Gao fetal SI+LI (H-new3) and Gao fetal LI vs colon+rectum (H-new3-debug); cross-platform effect-only</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>6 adult samples</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>14,537 epithelial cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>T1 bulk tumour support</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>TCGA COAD + READ</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Cancer Genome Atlas Network</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Nature, 2012</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>22810696</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>10.1038/nature11252</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>TCGA-COAD, TCGA-READ (GDC) via recount3</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq, recount3 Monorail, GENCODE v26 read counts</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Primary tumour vs solid-tissue normal, ~ tissue + project</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>624 tumours (458 COAD, 166 READ) / 51 normals</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>bulk_support annotation (no veto, plan v2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>T1 sensitivity</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>GTEx v8 colon</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>GTEx Consortium</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Science, 2020</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>32913098</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>10.1126/science.aaz1776</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>GTEx v8 (dbGaP phs000424) via recount3</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq, same recount3 pipeline</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>TCGA tumour vs GTEx Colon – Transverse; direction only (source confounded)</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>433 GTEx / 624 tumours</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Descriptive only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Processing resource</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>recount3</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Wilks C et al.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Genome Biol, 2021</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>34844637</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>10.1186/s13059-021-02533-6</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>duffel.rail.bio/recount3; R recount3 1.20.0</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>Uniform re-processing of TCGA + GTEx</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
         <is>
           <t>1,545 samples downloaded</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>Ensures TCGA/GTEx share one pipeline</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>S1 primary malignant epithelium</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Joanito CRC epithelial scRNA (5 cohorts: CRC-SG1, CRC-SG2, KUL3, KUL5, SMC)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Joanito I et al.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Nat Genet, 2022</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>35773407</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>10.1038/s41588-022-01100-4</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Synapse syn26844071 (counts syn26844072, metadata syn26844073, clinical syn39828015)</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>10x scRNA-seq, raw counts, GRCh38 Ensembl 93, symbols only; 49,155 epithelial cells</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>Author malignant (iCMS2/iCMS3, Tumor + Tumor-2) vs normal epithelium, ~ cohort + group</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>61 malignant / 24 normal patients</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Patient-level pseudobulks (≥ 50 cells); counts restricted</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Terms: non-commercial use; no transfer/disclosure of data or derived material</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>S2 epithelial replication + P progenitor check</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Pelka CRC immune-hub atlas</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Pelka K et al.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Cell, 2021</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>34450029</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>10.1016/j.cell.2021.08.003</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>GSE178341 (raw FASTQ: dbGaP phs002407)</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>10x scRNA-seq, raw counts, GPL16791; 370,115 cells</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>Tumour- vs normal-specimen epithelium (S2); tumour vs normal stem/TA cE01–03 (P)</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>62 tumour / 35 normal patients (P: 62 / 35)</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M17" s="5" t="inlineStr">
         <is>
           <t>Admitted; GEO release has no per-cell malignancy call</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M14"/>
+  <autoFilter ref="A1:M17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1464,51 +1665,51 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>In-house CRC Atlas</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Large-scale replication, gene–gene network (Fig 1F)</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Not available locally; PR/CRC-Atlas holds registry metadata only</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>FAP → adenoma → CRC progression (HTAN)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Disease-evolution validation</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Deferred; not used for discovery</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Joanito non-epithelial matrix (syn26844078, syn39828012)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Not required for S1</t>
         </is>

</xml_diff>

<commit_message>
docs: record benchmark v2 review — H-new2 cross-study human primary, Visium dropped
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -953,7 +953,7 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>GEO GEX/HTO pairing corrected by barcode overlap; hashtag samples can share a fetus</t>
+          <t>Human primary (cross-study) fetal arm (review 2026-10-02); GEO GEX/HTO pairing corrected by barcode overlap; hashtag samples can share a fetus</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>Adult n = 2 sections; fetal spots markedly less epithelial (composition confound)</t>
+          <t>Dropped from quantitative Step 2 (review 2026-10-02): composition-confounded, adult n = 2; failed QC record only</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>12,590 epithelial cells</t>
+          <t>Human primary (cross-study) with Fawkner fetal scRNA (review 2026-10-02); needs independent validation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
analysis: benchmark v2 addendum — primary-tissue bulk H-bulk1/H-bulk2 (Roadmap fetal SI vs HPA adult)
Both fail the frozen rule (TNFRSF12A fetal <= adult, panel not fetal-biased)
despite the OLFM4 maturation control. Evidence tiers recorded; registry,
31-marker summary, DATA records and docs updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not used or deferred'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1293,136 +1293,136 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>T1 bulk tumour support</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>TCGA COAD + READ</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Cancer Genome Atlas Network</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Nature, 2012</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>22810696</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>10.1038/nature11252</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2 (benchmark v2)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>H-bulk1/H-bulk2 fetal arm (tier B)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Roadmap fetal small intestine</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Roadmap Epigenomics Consortium (Kundaje A et al.); design per Finkbeiner SR et al., Stem Cell Rep 2015 (PMID 26050928)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Nature, 2015</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>25693563</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>10.1038/nature14248</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>TCGA-COAD, TCGA-READ (GDC) via recount3</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq, recount3 Monorail, GENCODE v26 read counts</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>Primary tumour vs solid-tissue normal, ~ tissue + project</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>624 tumours (458 COAD, 166 READ) / 51 normals</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>bulk_support annotation (no veto, plan v2)</t>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>GEO GSE18927 / SRA SRP001371 (GSM1059486, 507, 508, 517, 519, 521) via recount3</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Bulk total RNA-seq, whole tissue, recount3 counts</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Fetal SI 91–120 days vs HPA adult SI (H-bulk1) or duodenum (H-bulk2), edgeR ~ stage</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>6 fetal donors</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Tier B; same fetal samples in H-bulk1 and H-bulk2; library type differs from adult arm</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>T1 sensitivity</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>GTEx v8 colon</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>GTEx Consortium</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Science, 2020</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>32913098</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>10.1126/science.aaz1776</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2 (benchmark v2)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>H-bulk1/H-bulk2 adult arm (tier B)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>HPA adult small intestine / duodenum</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Fagerberg L et al.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Mol Cell Proteomics, 2014</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>24309898</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>10.1074/mcp.M113.035600</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>GTEx v8 (dbGaP phs000424) via recount3</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>Bulk RNA-seq, same recount3 pipeline</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>TCGA tumour vs GTEx Colon – Transverse; direction only (source confounded)</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>433 GTEx / 624 tumours</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
-        <is>
-          <t>Descriptive only</t>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>ArrayExpress E-MTAB-1733 / ENA ERP003613 via recount3</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Bulk poly(A) RNA-seq, whole tissue, 2 runs per sample summed</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Adult SI 4 + duodenum 2 (H-bulk1); duodenum 2 only (H-bulk2; Senger 2018 primary-tissue subset)</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>6 adult samples (H-bulk1) / 2 (H-bulk2)</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>Tier B; H-bulk2 not independent of H-bulk1</t>
         </is>
       </c>
     </row>
@@ -1434,32 +1434,32 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Processing resource</t>
+          <t>T1 bulk tumour support</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>recount3</t>
+          <t>TCGA COAD + READ</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Wilks C et al.</t>
+          <t>Cancer Genome Atlas Network</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Genome Biol, 2021</t>
+          <t>Nature, 2012</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>34844637</t>
+          <t>22810696</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>10.1186/s13059-021-02533-6</t>
+          <t>10.1038/nature11252</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1469,27 +1469,27 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>duffel.rail.bio/recount3; R recount3 1.20.0</t>
+          <t>TCGA-COAD, TCGA-READ (GDC) via recount3</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Uniform re-processing of TCGA + GTEx</t>
+          <t>Bulk RNA-seq, recount3 Monorail, GENCODE v26 read counts</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Primary tumour vs solid-tissue normal, ~ tissue + project</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>1,545 samples downloaded</t>
+          <t>624 tumours (458 COAD, 166 READ) / 51 normals</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Ensures TCGA/GTEx share one pipeline</t>
+          <t>bulk_support annotation (no veto, plan v2)</t>
         </is>
       </c>
     </row>
@@ -1501,32 +1501,32 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>S1 primary malignant epithelium</t>
+          <t>T1 sensitivity</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Joanito CRC epithelial scRNA (5 cohorts: CRC-SG1, CRC-SG2, KUL3, KUL5, SMC)</t>
+          <t>GTEx v8 colon</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Joanito I et al.</t>
+          <t>GTEx Consortium</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Nat Genet, 2022</t>
+          <t>Science, 2020</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>35773407</t>
+          <t>32913098</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>10.1038/s41588-022-01100-4</t>
+          <t>10.1126/science.aaz1776</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1536,27 +1536,27 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Synapse syn26844071 (counts syn26844072, metadata syn26844073, clinical syn39828015)</t>
+          <t>GTEx v8 (dbGaP phs000424) via recount3</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>10x scRNA-seq, raw counts, GRCh38 Ensembl 93, symbols only; 49,155 epithelial cells</t>
+          <t>Bulk RNA-seq, same recount3 pipeline</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>Author malignant (iCMS2/iCMS3, Tumor + Tumor-2) vs normal epithelium, ~ cohort + group</t>
+          <t>TCGA tumour vs GTEx Colon – Transverse; direction only (source confounded)</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Patient-level pseudobulks (≥ 50 cells); counts restricted</t>
+          <t>433 GTEx / 624 tumours</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Terms: non-commercial use; no transfer/disclosure of data or derived material</t>
+          <t>Descriptive only</t>
         </is>
       </c>
     </row>
@@ -1568,67 +1568,201 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>Processing resource</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>recount3</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Wilks C et al.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Genome Biol, 2021</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>34844637</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>10.1186/s13059-021-02533-6</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>duffel.rail.bio/recount3; R recount3 1.20.0</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Uniform re-processing of TCGA + GTEx</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>1,545 samples downloaded</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Ensures TCGA/GTEx share one pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>S1 primary malignant epithelium</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Joanito CRC epithelial scRNA (5 cohorts: CRC-SG1, CRC-SG2, KUL3, KUL5, SMC)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Joanito I et al.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Nat Genet, 2022</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>35773407</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>10.1038/s41588-022-01100-4</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Synapse syn26844071 (counts syn26844072, metadata syn26844073, clinical syn39828015)</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>10x scRNA-seq, raw counts, GRCh38 Ensembl 93, symbols only; 49,155 epithelial cells</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Author malignant (iCMS2/iCMS3, Tumor + Tumor-2) vs normal epithelium, ~ cohort + group</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Patient-level pseudobulks (≥ 50 cells); counts restricted</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Terms: non-commercial use; no transfer/disclosure of data or derived material</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
           <t>S2 epithelial replication + P progenitor check</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Pelka CRC immune-hub atlas</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Pelka K et al.</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Cell, 2021</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>34450029</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>10.1016/j.cell.2021.08.003</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>GSE178341 (raw FASTQ: dbGaP phs002407)</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>10x scRNA-seq, raw counts, GPL16791; 370,115 cells</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>Tumour- vs normal-specimen epithelium (S2); tumour vs normal stem/TA cE01–03 (P)</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
         <is>
           <t>62 tumour / 35 normal patients (P: 62 / 35)</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="M19" s="5" t="inlineStr">
         <is>
           <t>Admitted; GEO release has no per-cell malignancy call</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M17"/>
+  <autoFilter ref="A1:M19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
analysis: benchmark v2 addendum v1.2 — stage-resolved HGCA and Gao (early <9 W vs mid/late >=9 W)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -621,12 +621,12 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>16 fetal / 7 adult donors</t>
+          <t>16 fetal / 7 adult donors (6 &lt;9 PCW, 10 ≥9 PCW)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Invalidated (failed 31-marker biological QA)</t>
+          <t>Invalidated (failed 31-marker biological QA); stage-resolved (v1.2): early vs adult TNFRSF12A −1.58, mid/late vs adult −0.01, mid/late vs early +1.60 (P = 0.009); not promoted</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Invalidated with Step 2; fetal arm reused in benchmark v2 (H-new3, Gao-original recomputed)</t>
+          <t>Invalidated with Step 2; fetal arm reused in benchmark v2 (H-new3, Gao-original recomputed); stage-resolved (v1.2, &lt;9 / ≥9 W): mid/late vs adult TNFRSF12A −0.01 (GSE103154) / +0.69, P = 0.09, panel 20/24 (Wang); not promoted</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Failed marker benchmark (14/29 positive)</t>
+          <t>Failed marker benchmark (14/29 positive); not stage-splittable (all fetal 11–22.5 W GA ≥ 9 W)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(core): generated Methods references from provenance files; dataset registry final gate roles + Khaliq/Che/Tabula Sapiens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not used or deferred'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Invalidated (failed 31-marker biological QA); stage-resolved (v1.2): early vs adult TNFRSF12A −1.58, mid/late vs adult −0.01, mid/late vs early +1.60 (P = 0.009); not promoted</t>
+          <t>Invalidated (failed 31-marker biological QA); stage-resolved (v1.2): early vs adult TNFRSF12A −1.58, mid/late vs adult −0.01, mid/late vs early +1.60 (P = 0.009); not promoted; CIOC method v4.0: Gate H dataset (≥ 9 PCW arm: 10 fetal donors 9.2–17 PCW vs 7 adult donors, edgeR QL robust)</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Invalidated with Step 2; fetal arm reused in benchmark v2 (H-new3, Gao-original recomputed); stage-resolved (v1.2, &lt;9 / ≥9 W): mid/late vs adult TNFRSF12A −0.01 (GSE103154) / +0.69, P = 0.09, panel 20/24 (Wang); not promoted</t>
+          <t>Invalidated with Step 2; fetal arm reused in benchmark v2 (H-new3, Gao-original recomputed); stage-resolved (v1.2, &lt;9 / ≥9 W): mid/late vs adult TNFRSF12A −0.01 (GSE103154) / +0.69, P = 0.09, panel 20/24 (Wang); not promoted; CIOC method v4.0: Gate H dataset (Gao-original ≥ 9 W: fetal LI epithelium, 7 embryos 9–25 W, vs GSE103154 adult LI P1/P2; cross-platform effect-only, Welch P descriptive)</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Invalidated with Step 2</t>
+          <t>Invalidated with Step 2; CIOC method v4.0: Gate M dataset (3 vs 3, edgeR QL robust)</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>In vivo replication only (10/23 positive)</t>
+          <t>In vivo replication only (10/23 positive); CIOC method v4.0: supportive replication flag only (not selecting)</t>
         </is>
       </c>
     </row>
@@ -1761,8 +1761,209 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>3 (Extended CIOC)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Gate E + coherence, primary</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Khaliq CRC single-cell atlas</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Khaliq AM et al.</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Genome Biol, 2022</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>35538548</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>10.1186/s13059-022-02677-z</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>GSE200997</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>10x scRNA-seq, raw UMI CSV (no cell types deposited)</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Tumour-derived epithelial vs other compartments; within-sample CIOC coherence</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>16 CRC + 7 adjacent normal samples (16 patients); tumour samples used; 8 coherence strata (≥ 200 epithelial cells)</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Compartments annotated in-house (marker-module detection); malignancy not inferred; refinement-stage replication, not external validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>3 (Extended CIOC)</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Gate E + coherence, replication</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Che CRC + liver-metastasis atlas</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Che LH et al.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Cell Discov, 2021</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>34489408</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>10.1038/s41421-021-00312-y</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>GSE178318</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>10x scRNA-seq, MTX (no cell annotation)</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>As Khaliq</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>6 patients, primary CRC + liver metastasis (PBMC excluded); 8 coherence strata</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Includes patients with preoperative chemotherapy; compartments annotated in-house; refinement-stage replication</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>3 (Extended CIOC)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Compartment annotation only</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Tabula Sapiens large intestine</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Tabula Sapiens Consortium</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Science, 2022</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>35549404</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>10.1126/science.abl4896</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>figshare 10.6084/m9.figshare.14267219 (TS_Large_Intestine)</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>10x scRNA-seq (raw_counts layer)</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Adult normal epithelial vs top non-epithelial compartment</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>2 donors</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Annotation only; never selecting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M19"/>
+  <autoFilter ref="A1:M22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
analysis(core): supplementary tissue/cancer breadth annotation (Cao 2020 fetal atlas; Toil TCGA+GTEx) applied once; restricted outputs git-ignored
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not used or deferred'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1962,8 +1962,142 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Breadth annotation</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Fetal tissue breadth (annotation only)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Cao fetal atlas (sci-RNA-seq3)</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Cao J et al.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Science, 2020</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>33184181</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>10.1126/science.aba7721</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>GSE156793 (S1, S2, S4–S7 aggregated tables)</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>sci-RNA-seq3; organ × cell-type pseudobulk CPM</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Organ-epithelium expression across 8 fetal organs (72–129 days post-conception)</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Aggregated across fetuses; intestine/stomach/pancreas/kidney whole-cell, lung/liver/placenta/thymus nuclei</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Annotation only; never selecting (BREADTH_ANNOTATION_PLAN.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Breadth annotation</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Cancer reactivation breadth (annotation only)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>UCSC Toil TCGA + GTEx</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Vivian J et al.</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Nat Biotechnol, 2017</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>28398314</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>10.1038/nbt.3772</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>UCSC Xena toil hub: TcgaTargetGtex_rsem_gene_tpm, TcgaTargetGTEX_phenotype</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Bulk RNA-seq, uniform RSEM TPM</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>21 TCGA carcinoma types vs GTEx matched tissue + TCGA solid-tissue normal</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>21 eligible carcinomas (≥ 10 tumour, ≥ 10 normal)</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>Annotation only; bulk composition and GTEx/TCGA batch caveats</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M22"/>
+  <autoFilter ref="A1:M24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
analysis(core): pan-cancer breadth of CIOC reactivation in bulk tumours (annotation v2, applied once); fetal tissue breadth moved to internal exploration
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -1965,12 +1965,12 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Breadth annotation</t>
+          <t>Exploratory only (not a deliverable)</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Fetal tissue breadth (annotation only)</t>
+          <t>Fetal tissue breadth (superseded by breadth plan v2)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: dataset registry — add Kang 2024 pan-cancer atlas and HGNC; Toil relabelled secondary; draft pan-cancer epithelial plan + extraction script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DATASET_REGISTRY.xlsx
+++ b/docs/DATASET_REGISTRY.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Datasets'!$A$1:$M$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Not used or deferred'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2032,12 +2032,12 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Breadth annotation</t>
+          <t>Breadth annotation (secondary)</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Cancer reactivation breadth (annotation only)</t>
+          <t>Bulk cancer breadth; downgraded to secondary annotation (composition-confounded)</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2096,8 +2096,142 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Pan-cancer epithelial annotation (primary)</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Malignant vs normal epithelial reactivation across carcinomas</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Kang pan-cancer tumour–normal scRNA atlas</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Kang J et al.</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Nat Commun, 2024</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>38744958</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>10.1038/s41467-024-48310-4</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Zenodo 10.5281/zenodo.10651059 (atlas_dataset.tar, md5 2d78f5de610538ed01af6338fc312f27; Documentation for scRNA-seq dataset.xlsx)</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>scRNA-seq meta-atlas; per-dataset log1p(CP10k) h5ad with authors' cell types and inferCNVpy malignant call</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>CNV-inferred malignant epithelial vs normal epithelial (adjacent or healthy), patient pseudobulk</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>104 datasets, 30 cancer types, 1,070 tumour / 493 normal samples, 999 donors</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>Excluded for independence: crc_HOLee_GSE132465, crc_HOLee_GSE144735, crc_HOLee_GSE132257, crc_meta_GSE178318, intestine_gca, crc_pan_blueprint; download in progress (2026-10-05); plan core_oncofetal/docs/PANCANCER_EPITHELIAL_PLAN.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Processing resource</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Gene-symbol resolution (all modules)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>HGNC gene ID mapping</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Seal RL et al.</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Nucleic Acids Res, 2023</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>36243972</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>10.1093/nar/gkac888</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Human</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>genenames.org custom download (access 2026-08-13)</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Reference table</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Approved, previous and alias symbols; Ensembl IDs</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>Used for CCN2/CTGF-type symbol resolution and Ensembl-ID mapping (feature audit, atlases, Toil, Kang)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M24"/>
+  <autoFilter ref="A1:M26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>